<commit_message>
feat: add fine-tuned model to benchmark suite and include datasets in project directory
</commit_message>
<xml_diff>
--- a/benchmark_results.xlsx
+++ b/benchmark_results.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>Model Name</t>
   </si>
@@ -55,10 +55,16 @@
     <t>Pruned</t>
   </si>
   <si>
+    <t>Fine-tuned-50epochs</t>
+  </si>
+  <si>
     <t>yolov5s.pt</t>
   </si>
   <si>
     <t>yolov5s-pruned.pt</t>
+  </si>
+  <si>
+    <t>runs/train/exp15/weights/best.pt</t>
   </si>
 </sst>
 </file>
@@ -416,7 +422,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
@@ -459,7 +465,7 @@
         <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C2">
         <v>7225885</v>
@@ -480,13 +486,13 @@
         <v>0.361</v>
       </c>
       <c r="I2">
-        <v>1.22</v>
+        <v>1.27</v>
       </c>
       <c r="J2">
-        <v>1.06</v>
+        <v>1.21</v>
       </c>
       <c r="K2">
-        <v>2.28</v>
+        <v>2.48</v>
       </c>
     </row>
     <row r="3" spans="1:11">
@@ -494,7 +500,7 @@
         <v>12</v>
       </c>
       <c r="B3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C3">
         <v>5933813</v>
@@ -515,13 +521,48 @@
         <v>0.2316</v>
       </c>
       <c r="I3">
-        <v>1.14</v>
+        <v>1.17</v>
       </c>
       <c r="J3">
-        <v>0.96</v>
+        <v>1.08</v>
       </c>
       <c r="K3">
-        <v>2.09</v>
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11">
+      <c r="A4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4">
+        <v>5933813</v>
+      </c>
+      <c r="D4">
+        <v>14.317</v>
+      </c>
+      <c r="E4">
+        <v>0.5855</v>
+      </c>
+      <c r="F4">
+        <v>0.4301</v>
+      </c>
+      <c r="G4">
+        <v>0.4433</v>
+      </c>
+      <c r="H4">
+        <v>0.2679</v>
+      </c>
+      <c r="I4">
+        <v>1.17</v>
+      </c>
+      <c r="J4">
+        <v>1.4</v>
+      </c>
+      <c r="K4">
+        <v>2.58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactor: implement robust parameter/FLOPS selection logic and enhance benchmark visualization with new plotting and export utilities.
</commit_message>
<xml_diff>
--- a/benchmark_results.xlsx
+++ b/benchmark_results.xlsx
@@ -64,23 +64,15 @@
     <t>yolov5s-pruned.pt</t>
   </si>
   <si>
-    <t>runs/train/exp15/weights/best.pt</t>
+    <t>yolov5s-pruned-finetuned.pt</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -96,7 +88,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -104,30 +96,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -426,37 +400,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -474,25 +448,25 @@
         <v>16.436</v>
       </c>
       <c r="E2">
-        <v>0.6645</v>
+        <v>0.6542</v>
       </c>
       <c r="F2">
-        <v>0.5239</v>
+        <v>0.5532</v>
       </c>
       <c r="G2">
-        <v>0.5634</v>
+        <v>0.5987</v>
       </c>
       <c r="H2">
-        <v>0.361</v>
+        <v>0.4004</v>
       </c>
       <c r="I2">
-        <v>1.27</v>
+        <v>101.54</v>
       </c>
       <c r="J2">
-        <v>1.21</v>
+        <v>4.73</v>
       </c>
       <c r="K2">
-        <v>2.48</v>
+        <v>106.27</v>
       </c>
     </row>
     <row r="3" spans="1:11">
@@ -509,25 +483,25 @@
         <v>14.317</v>
       </c>
       <c r="E3">
-        <v>0.6163999999999999</v>
+        <v>0.6128</v>
       </c>
       <c r="F3">
-        <v>0.3686</v>
+        <v>0.3902</v>
       </c>
       <c r="G3">
-        <v>0.4037</v>
+        <v>0.4388</v>
       </c>
       <c r="H3">
-        <v>0.2316</v>
+        <v>0.2575</v>
       </c>
       <c r="I3">
-        <v>1.17</v>
+        <v>96.95999999999999</v>
       </c>
       <c r="J3">
-        <v>1.08</v>
+        <v>3.24</v>
       </c>
       <c r="K3">
-        <v>2.25</v>
+        <v>100.2</v>
       </c>
     </row>
     <row r="4" spans="1:11">
@@ -544,25 +518,25 @@
         <v>14.317</v>
       </c>
       <c r="E4">
-        <v>0.5855</v>
+        <v>0.6404</v>
       </c>
       <c r="F4">
-        <v>0.4301</v>
+        <v>0.4123</v>
       </c>
       <c r="G4">
-        <v>0.4433</v>
+        <v>0.4606</v>
       </c>
       <c r="H4">
-        <v>0.2679</v>
+        <v>0.2909</v>
       </c>
       <c r="I4">
-        <v>1.17</v>
+        <v>97.36</v>
       </c>
       <c r="J4">
-        <v>1.4</v>
+        <v>11.04</v>
       </c>
       <c r="K4">
-        <v>2.58</v>
+        <v>108.41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>